<commit_message>
Add Training & Competency module (certificate/licence expiry)
New Training & Competency page: per-person competency records (inductions,
statutory licences, medicals, skills) with expiry tracking and Valid/Expiring/
Expired status. KPI cards (currency %), currency-by-department and records-by-
type charts, and a register sorted soonest-to-expire. Expiring/expired statutory
licences and medicals now raise alerts. Sample competency.xlsx (198 rows) added.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/activity_log.xlsx
+++ b/data/activity_log.xlsx
@@ -509,7 +509,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -568,7 +568,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -745,7 +745,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -863,7 +863,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -981,7 +981,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1099,7 +1099,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1217,7 +1217,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1512,7 +1512,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1571,7 +1571,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1630,7 +1630,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1689,7 +1689,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1866,7 +1866,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1925,7 +1925,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1984,7 +1984,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2102,7 +2102,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2161,7 +2161,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2220,7 +2220,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2279,7 +2279,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2338,7 +2338,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2397,7 +2397,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2456,7 +2456,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -2574,7 +2574,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -2633,7 +2633,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2751,7 +2751,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -2869,7 +2869,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2928,7 +2928,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2987,7 +2987,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3046,7 +3046,7 @@
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -3105,7 +3105,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -3164,7 +3164,7 @@
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -3282,7 +3282,7 @@
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -3341,7 +3341,7 @@
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -3459,7 +3459,7 @@
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -3518,7 +3518,7 @@
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -3577,7 +3577,7 @@
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -3636,7 +3636,7 @@
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -3695,7 +3695,7 @@
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -3754,7 +3754,7 @@
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -3813,7 +3813,7 @@
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -3872,7 +3872,7 @@
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -3931,7 +3931,7 @@
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -3990,7 +3990,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -4049,7 +4049,7 @@
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -4167,7 +4167,7 @@
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -4226,7 +4226,7 @@
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -4344,7 +4344,7 @@
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -4403,7 +4403,7 @@
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -4462,7 +4462,7 @@
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -4521,7 +4521,7 @@
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -4580,7 +4580,7 @@
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -4639,7 +4639,7 @@
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -4757,7 +4757,7 @@
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -4816,7 +4816,7 @@
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -4875,7 +4875,7 @@
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -4934,7 +4934,7 @@
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -4993,7 +4993,7 @@
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -5052,7 +5052,7 @@
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -5111,7 +5111,7 @@
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -5170,7 +5170,7 @@
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -5229,7 +5229,7 @@
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -5288,7 +5288,7 @@
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -5406,7 +5406,7 @@
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -5465,7 +5465,7 @@
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -5524,7 +5524,7 @@
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -5701,7 +5701,7 @@
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -5760,7 +5760,7 @@
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -5819,7 +5819,7 @@
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -5878,7 +5878,7 @@
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -5937,7 +5937,7 @@
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -5996,7 +5996,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -6055,7 +6055,7 @@
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -6114,7 +6114,7 @@
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -6232,7 +6232,7 @@
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -6291,7 +6291,7 @@
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -6350,7 +6350,7 @@
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -6409,7 +6409,7 @@
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -6468,7 +6468,7 @@
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -6645,7 +6645,7 @@
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -6704,7 +6704,7 @@
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -6763,7 +6763,7 @@
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -6822,7 +6822,7 @@
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -6881,7 +6881,7 @@
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -6940,7 +6940,7 @@
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -6999,7 +6999,7 @@
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -7058,7 +7058,7 @@
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -7117,7 +7117,7 @@
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -7176,7 +7176,7 @@
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -7235,7 +7235,7 @@
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -7294,7 +7294,7 @@
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -7353,7 +7353,7 @@
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -7412,7 +7412,7 @@
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -7471,7 +7471,7 @@
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -7530,7 +7530,7 @@
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -7589,7 +7589,7 @@
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -7707,7 +7707,7 @@
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -7766,7 +7766,7 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -7825,7 +7825,7 @@
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -7884,7 +7884,7 @@
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -7943,7 +7943,7 @@
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -8002,7 +8002,7 @@
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -8061,7 +8061,7 @@
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -8120,7 +8120,7 @@
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -8238,7 +8238,7 @@
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -8297,7 +8297,7 @@
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -8356,7 +8356,7 @@
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -8415,7 +8415,7 @@
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -8474,7 +8474,7 @@
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -8533,7 +8533,7 @@
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -8592,7 +8592,7 @@
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -8651,7 +8651,7 @@
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -8710,7 +8710,7 @@
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -8769,7 +8769,7 @@
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -8828,7 +8828,7 @@
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -8887,7 +8887,7 @@
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -8946,7 +8946,7 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -9005,7 +9005,7 @@
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -9064,7 +9064,7 @@
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -9123,7 +9123,7 @@
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -9182,7 +9182,7 @@
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -9241,7 +9241,7 @@
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -9300,7 +9300,7 @@
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -9359,7 +9359,7 @@
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -9418,7 +9418,7 @@
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -9477,7 +9477,7 @@
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -9536,7 +9536,7 @@
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -9595,7 +9595,7 @@
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -9654,7 +9654,7 @@
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -9713,7 +9713,7 @@
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -9772,7 +9772,7 @@
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -9831,7 +9831,7 @@
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -9890,7 +9890,7 @@
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -9949,7 +9949,7 @@
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -10008,7 +10008,7 @@
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -10067,7 +10067,7 @@
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -10126,7 +10126,7 @@
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -10185,7 +10185,7 @@
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -10244,7 +10244,7 @@
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -10303,7 +10303,7 @@
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -10362,7 +10362,7 @@
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -10421,7 +10421,7 @@
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -10480,7 +10480,7 @@
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -10539,7 +10539,7 @@
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -10598,7 +10598,7 @@
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -10657,7 +10657,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -10716,7 +10716,7 @@
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -10775,7 +10775,7 @@
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -10834,7 +10834,7 @@
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -10893,7 +10893,7 @@
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -10952,7 +10952,7 @@
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -11011,7 +11011,7 @@
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -11070,7 +11070,7 @@
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -11129,7 +11129,7 @@
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -11247,7 +11247,7 @@
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -11306,7 +11306,7 @@
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -11365,7 +11365,7 @@
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -11424,7 +11424,7 @@
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -11483,7 +11483,7 @@
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -11542,7 +11542,7 @@
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -11601,7 +11601,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -11660,7 +11660,7 @@
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -11719,7 +11719,7 @@
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -11778,7 +11778,7 @@
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -11837,7 +11837,7 @@
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -11896,7 +11896,7 @@
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -11955,7 +11955,7 @@
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -12014,7 +12014,7 @@
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -12073,7 +12073,7 @@
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -12132,7 +12132,7 @@
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -12191,7 +12191,7 @@
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -12250,7 +12250,7 @@
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -12309,7 +12309,7 @@
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -12368,7 +12368,7 @@
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -12427,7 +12427,7 @@
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -12486,7 +12486,7 @@
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -12545,7 +12545,7 @@
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -12604,7 +12604,7 @@
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -12663,7 +12663,7 @@
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -12722,7 +12722,7 @@
     </row>
     <row r="209">
       <c r="A209" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
     </row>
     <row r="210">
       <c r="A210" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -12840,7 +12840,7 @@
     </row>
     <row r="211">
       <c r="A211" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -12899,7 +12899,7 @@
     </row>
     <row r="212">
       <c r="A212" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
@@ -12958,7 +12958,7 @@
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
@@ -13017,7 +13017,7 @@
     </row>
     <row r="214">
       <c r="A214" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -13076,7 +13076,7 @@
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -13135,7 +13135,7 @@
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
@@ -13194,7 +13194,7 @@
     </row>
     <row r="217">
       <c r="A217" s="1" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -13253,7 +13253,7 @@
     </row>
     <row r="218">
       <c r="A218" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -13312,7 +13312,7 @@
     </row>
     <row r="219">
       <c r="A219" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -13371,7 +13371,7 @@
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -13430,7 +13430,7 @@
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -13489,7 +13489,7 @@
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -13548,7 +13548,7 @@
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -13607,7 +13607,7 @@
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -13666,7 +13666,7 @@
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -13725,7 +13725,7 @@
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -13784,7 +13784,7 @@
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -13843,7 +13843,7 @@
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -13902,7 +13902,7 @@
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -13961,7 +13961,7 @@
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -14020,7 +14020,7 @@
     </row>
     <row r="231">
       <c r="A231" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -14079,7 +14079,7 @@
     </row>
     <row r="232">
       <c r="A232" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
@@ -14138,7 +14138,7 @@
     </row>
     <row r="233">
       <c r="A233" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -14197,7 +14197,7 @@
     </row>
     <row r="234">
       <c r="A234" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -14256,7 +14256,7 @@
     </row>
     <row r="235">
       <c r="A235" s="1" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -14315,7 +14315,7 @@
     </row>
     <row r="236">
       <c r="A236" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
@@ -14374,7 +14374,7 @@
     </row>
     <row r="237">
       <c r="A237" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
@@ -14433,7 +14433,7 @@
     </row>
     <row r="238">
       <c r="A238" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
@@ -14492,7 +14492,7 @@
     </row>
     <row r="239">
       <c r="A239" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
@@ -14551,7 +14551,7 @@
     </row>
     <row r="240">
       <c r="A240" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
@@ -14610,7 +14610,7 @@
     </row>
     <row r="241">
       <c r="A241" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
@@ -14669,7 +14669,7 @@
     </row>
     <row r="242">
       <c r="A242" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
@@ -14728,7 +14728,7 @@
     </row>
     <row r="243">
       <c r="A243" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
@@ -14787,7 +14787,7 @@
     </row>
     <row r="244">
       <c r="A244" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
@@ -14846,7 +14846,7 @@
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
@@ -14905,7 +14905,7 @@
     </row>
     <row r="246">
       <c r="A246" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
@@ -14964,7 +14964,7 @@
     </row>
     <row r="247">
       <c r="A247" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
@@ -15023,7 +15023,7 @@
     </row>
     <row r="248">
       <c r="A248" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
@@ -15082,7 +15082,7 @@
     </row>
     <row r="249">
       <c r="A249" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
@@ -15141,7 +15141,7 @@
     </row>
     <row r="250">
       <c r="A250" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B250" t="inlineStr">
         <is>
@@ -15200,7 +15200,7 @@
     </row>
     <row r="251">
       <c r="A251" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B251" t="inlineStr">
         <is>
@@ -15259,7 +15259,7 @@
     </row>
     <row r="252">
       <c r="A252" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B252" t="inlineStr">
         <is>
@@ -15318,7 +15318,7 @@
     </row>
     <row r="253">
       <c r="A253" s="1" t="n">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B253" t="inlineStr">
         <is>
@@ -15377,7 +15377,7 @@
     </row>
     <row r="254">
       <c r="A254" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
@@ -15436,7 +15436,7 @@
     </row>
     <row r="255">
       <c r="A255" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
@@ -15495,7 +15495,7 @@
     </row>
     <row r="256">
       <c r="A256" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
@@ -15554,7 +15554,7 @@
     </row>
     <row r="257">
       <c r="A257" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
@@ -15613,7 +15613,7 @@
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
@@ -15672,7 +15672,7 @@
     </row>
     <row r="259">
       <c r="A259" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
@@ -15731,7 +15731,7 @@
     </row>
     <row r="260">
       <c r="A260" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B260" t="inlineStr">
         <is>
@@ -15790,7 +15790,7 @@
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B261" t="inlineStr">
         <is>
@@ -15849,7 +15849,7 @@
     </row>
     <row r="262">
       <c r="A262" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B262" t="inlineStr">
         <is>
@@ -15908,7 +15908,7 @@
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B263" t="inlineStr">
         <is>
@@ -15967,7 +15967,7 @@
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B264" t="inlineStr">
         <is>
@@ -16026,7 +16026,7 @@
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B265" t="inlineStr">
         <is>
@@ -16085,7 +16085,7 @@
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B266" t="inlineStr">
         <is>
@@ -16144,7 +16144,7 @@
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B267" t="inlineStr">
         <is>
@@ -16203,7 +16203,7 @@
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B268" t="inlineStr">
         <is>
@@ -16262,7 +16262,7 @@
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B269" t="inlineStr">
         <is>
@@ -16321,7 +16321,7 @@
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
@@ -16380,7 +16380,7 @@
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
@@ -16439,7 +16439,7 @@
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
@@ -16498,7 +16498,7 @@
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
@@ -16557,7 +16557,7 @@
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
@@ -16616,7 +16616,7 @@
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
@@ -16675,7 +16675,7 @@
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
@@ -16734,7 +16734,7 @@
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
@@ -16793,7 +16793,7 @@
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
@@ -16852,7 +16852,7 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
@@ -16911,7 +16911,7 @@
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
@@ -16970,7 +16970,7 @@
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
@@ -17029,7 +17029,7 @@
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
@@ -17088,7 +17088,7 @@
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
@@ -17147,7 +17147,7 @@
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
@@ -17206,7 +17206,7 @@
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
@@ -17265,7 +17265,7 @@
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
@@ -17324,7 +17324,7 @@
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
@@ -17383,7 +17383,7 @@
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
@@ -17442,7 +17442,7 @@
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
-        <v>45901</v>
+        <v>45931</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
@@ -17501,7 +17501,7 @@
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
@@ -17560,7 +17560,7 @@
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
@@ -17619,7 +17619,7 @@
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
@@ -17678,7 +17678,7 @@
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B293" t="inlineStr">
         <is>
@@ -17737,7 +17737,7 @@
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B294" t="inlineStr">
         <is>
@@ -17796,7 +17796,7 @@
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
@@ -17855,7 +17855,7 @@
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B296" t="inlineStr">
         <is>
@@ -17914,7 +17914,7 @@
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B297" t="inlineStr">
         <is>
@@ -17973,7 +17973,7 @@
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B298" t="inlineStr">
         <is>
@@ -18032,7 +18032,7 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B299" t="inlineStr">
         <is>
@@ -18091,7 +18091,7 @@
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B300" t="inlineStr">
         <is>
@@ -18150,7 +18150,7 @@
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B301" t="inlineStr">
         <is>
@@ -18209,7 +18209,7 @@
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B302" t="inlineStr">
         <is>
@@ -18268,7 +18268,7 @@
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B303" t="inlineStr">
         <is>
@@ -18327,7 +18327,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B304" t="inlineStr">
         <is>
@@ -18386,7 +18386,7 @@
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B305" t="inlineStr">
         <is>
@@ -18445,7 +18445,7 @@
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B306" t="inlineStr">
         <is>
@@ -18504,7 +18504,7 @@
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B307" t="inlineStr">
         <is>
@@ -18563,7 +18563,7 @@
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B308" t="inlineStr">
         <is>
@@ -18622,7 +18622,7 @@
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B309" t="inlineStr">
         <is>
@@ -18681,7 +18681,7 @@
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B310" t="inlineStr">
         <is>
@@ -18740,7 +18740,7 @@
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B311" t="inlineStr">
         <is>
@@ -18799,7 +18799,7 @@
     </row>
     <row r="312">
       <c r="A312" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B312" t="inlineStr">
         <is>
@@ -18858,7 +18858,7 @@
     </row>
     <row r="313">
       <c r="A313" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B313" t="inlineStr">
         <is>
@@ -18917,7 +18917,7 @@
     </row>
     <row r="314">
       <c r="A314" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B314" t="inlineStr">
         <is>
@@ -18976,7 +18976,7 @@
     </row>
     <row r="315">
       <c r="A315" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B315" t="inlineStr">
         <is>
@@ -19035,7 +19035,7 @@
     </row>
     <row r="316">
       <c r="A316" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B316" t="inlineStr">
         <is>
@@ -19094,7 +19094,7 @@
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B317" t="inlineStr">
         <is>
@@ -19153,7 +19153,7 @@
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B318" t="inlineStr">
         <is>
@@ -19212,7 +19212,7 @@
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B319" t="inlineStr">
         <is>
@@ -19271,7 +19271,7 @@
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B320" t="inlineStr">
         <is>
@@ -19330,7 +19330,7 @@
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B321" t="inlineStr">
         <is>
@@ -19389,7 +19389,7 @@
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B322" t="inlineStr">
         <is>
@@ -19448,7 +19448,7 @@
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B323" t="inlineStr">
         <is>
@@ -19507,7 +19507,7 @@
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B324" t="inlineStr">
         <is>
@@ -19566,7 +19566,7 @@
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B325" t="inlineStr">
         <is>
@@ -19625,7 +19625,7 @@
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B326" t="inlineStr">
         <is>
@@ -19684,7 +19684,7 @@
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B327" t="inlineStr">
         <is>
@@ -19743,7 +19743,7 @@
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B328" t="inlineStr">
         <is>
@@ -19802,7 +19802,7 @@
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B329" t="inlineStr">
         <is>
@@ -19861,7 +19861,7 @@
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B330" t="inlineStr">
         <is>
@@ -19920,7 +19920,7 @@
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B331" t="inlineStr">
         <is>
@@ -19979,7 +19979,7 @@
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B332" t="inlineStr">
         <is>
@@ -20038,7 +20038,7 @@
     </row>
     <row r="333">
       <c r="A333" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B333" t="inlineStr">
         <is>
@@ -20097,7 +20097,7 @@
     </row>
     <row r="334">
       <c r="A334" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B334" t="inlineStr">
         <is>
@@ -20156,7 +20156,7 @@
     </row>
     <row r="335">
       <c r="A335" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B335" t="inlineStr">
         <is>
@@ -20215,7 +20215,7 @@
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B336" t="inlineStr">
         <is>
@@ -20274,7 +20274,7 @@
     </row>
     <row r="337">
       <c r="A337" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B337" t="inlineStr">
         <is>
@@ -20333,7 +20333,7 @@
     </row>
     <row r="338">
       <c r="A338" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B338" t="inlineStr">
         <is>
@@ -20392,7 +20392,7 @@
     </row>
     <row r="339">
       <c r="A339" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B339" t="inlineStr">
         <is>
@@ -20451,7 +20451,7 @@
     </row>
     <row r="340">
       <c r="A340" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B340" t="inlineStr">
         <is>
@@ -20510,7 +20510,7 @@
     </row>
     <row r="341">
       <c r="A341" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B341" t="inlineStr">
         <is>
@@ -20569,7 +20569,7 @@
     </row>
     <row r="342">
       <c r="A342" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B342" t="inlineStr">
         <is>
@@ -20628,7 +20628,7 @@
     </row>
     <row r="343">
       <c r="A343" s="1" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B343" t="inlineStr">
         <is>
@@ -20687,7 +20687,7 @@
     </row>
     <row r="344">
       <c r="A344" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B344" t="inlineStr">
         <is>
@@ -20746,7 +20746,7 @@
     </row>
     <row r="345">
       <c r="A345" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B345" t="inlineStr">
         <is>
@@ -20805,7 +20805,7 @@
     </row>
     <row r="346">
       <c r="A346" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B346" t="inlineStr">
         <is>
@@ -20864,7 +20864,7 @@
     </row>
     <row r="347">
       <c r="A347" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B347" t="inlineStr">
         <is>
@@ -20923,7 +20923,7 @@
     </row>
     <row r="348">
       <c r="A348" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B348" t="inlineStr">
         <is>
@@ -20982,7 +20982,7 @@
     </row>
     <row r="349">
       <c r="A349" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B349" t="inlineStr">
         <is>
@@ -21041,7 +21041,7 @@
     </row>
     <row r="350">
       <c r="A350" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B350" t="inlineStr">
         <is>
@@ -21100,7 +21100,7 @@
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B351" t="inlineStr">
         <is>
@@ -21159,7 +21159,7 @@
     </row>
     <row r="352">
       <c r="A352" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B352" t="inlineStr">
         <is>
@@ -21218,7 +21218,7 @@
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B353" t="inlineStr">
         <is>
@@ -21277,7 +21277,7 @@
     </row>
     <row r="354">
       <c r="A354" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B354" t="inlineStr">
         <is>
@@ -21336,7 +21336,7 @@
     </row>
     <row r="355">
       <c r="A355" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B355" t="inlineStr">
         <is>
@@ -21395,7 +21395,7 @@
     </row>
     <row r="356">
       <c r="A356" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B356" t="inlineStr">
         <is>
@@ -21454,7 +21454,7 @@
     </row>
     <row r="357">
       <c r="A357" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B357" t="inlineStr">
         <is>
@@ -21513,7 +21513,7 @@
     </row>
     <row r="358">
       <c r="A358" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B358" t="inlineStr">
         <is>
@@ -21572,7 +21572,7 @@
     </row>
     <row r="359">
       <c r="A359" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B359" t="inlineStr">
         <is>
@@ -21631,7 +21631,7 @@
     </row>
     <row r="360">
       <c r="A360" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B360" t="inlineStr">
         <is>
@@ -21690,7 +21690,7 @@
     </row>
     <row r="361">
       <c r="A361" s="1" t="n">
-        <v>46023</v>
+        <v>46054</v>
       </c>
       <c r="B361" t="inlineStr">
         <is>
@@ -21749,7 +21749,7 @@
     </row>
     <row r="362">
       <c r="A362" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B362" t="inlineStr">
         <is>
@@ -21808,7 +21808,7 @@
     </row>
     <row r="363">
       <c r="A363" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B363" t="inlineStr">
         <is>
@@ -21867,7 +21867,7 @@
     </row>
     <row r="364">
       <c r="A364" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B364" t="inlineStr">
         <is>
@@ -21926,7 +21926,7 @@
     </row>
     <row r="365">
       <c r="A365" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B365" t="inlineStr">
         <is>
@@ -21985,7 +21985,7 @@
     </row>
     <row r="366">
       <c r="A366" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B366" t="inlineStr">
         <is>
@@ -22044,7 +22044,7 @@
     </row>
     <row r="367">
       <c r="A367" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B367" t="inlineStr">
         <is>
@@ -22103,7 +22103,7 @@
     </row>
     <row r="368">
       <c r="A368" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B368" t="inlineStr">
         <is>
@@ -22162,7 +22162,7 @@
     </row>
     <row r="369">
       <c r="A369" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B369" t="inlineStr">
         <is>
@@ -22221,7 +22221,7 @@
     </row>
     <row r="370">
       <c r="A370" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B370" t="inlineStr">
         <is>
@@ -22280,7 +22280,7 @@
     </row>
     <row r="371">
       <c r="A371" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B371" t="inlineStr">
         <is>
@@ -22339,7 +22339,7 @@
     </row>
     <row r="372">
       <c r="A372" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B372" t="inlineStr">
         <is>
@@ -22398,7 +22398,7 @@
     </row>
     <row r="373">
       <c r="A373" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B373" t="inlineStr">
         <is>
@@ -22457,7 +22457,7 @@
     </row>
     <row r="374">
       <c r="A374" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B374" t="inlineStr">
         <is>
@@ -22516,7 +22516,7 @@
     </row>
     <row r="375">
       <c r="A375" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B375" t="inlineStr">
         <is>
@@ -22575,7 +22575,7 @@
     </row>
     <row r="376">
       <c r="A376" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B376" t="inlineStr">
         <is>
@@ -22634,7 +22634,7 @@
     </row>
     <row r="377">
       <c r="A377" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B377" t="inlineStr">
         <is>
@@ -22693,7 +22693,7 @@
     </row>
     <row r="378">
       <c r="A378" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B378" t="inlineStr">
         <is>
@@ -22752,7 +22752,7 @@
     </row>
     <row r="379">
       <c r="A379" s="1" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B379" t="inlineStr">
         <is>
@@ -22811,7 +22811,7 @@
     </row>
     <row r="380">
       <c r="A380" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B380" t="inlineStr">
         <is>
@@ -22870,7 +22870,7 @@
     </row>
     <row r="381">
       <c r="A381" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B381" t="inlineStr">
         <is>
@@ -22929,7 +22929,7 @@
     </row>
     <row r="382">
       <c r="A382" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B382" t="inlineStr">
         <is>
@@ -22988,7 +22988,7 @@
     </row>
     <row r="383">
       <c r="A383" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B383" t="inlineStr">
         <is>
@@ -23047,7 +23047,7 @@
     </row>
     <row r="384">
       <c r="A384" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B384" t="inlineStr">
         <is>
@@ -23106,7 +23106,7 @@
     </row>
     <row r="385">
       <c r="A385" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B385" t="inlineStr">
         <is>
@@ -23165,7 +23165,7 @@
     </row>
     <row r="386">
       <c r="A386" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B386" t="inlineStr">
         <is>
@@ -23224,7 +23224,7 @@
     </row>
     <row r="387">
       <c r="A387" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B387" t="inlineStr">
         <is>
@@ -23283,7 +23283,7 @@
     </row>
     <row r="388">
       <c r="A388" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B388" t="inlineStr">
         <is>
@@ -23342,7 +23342,7 @@
     </row>
     <row r="389">
       <c r="A389" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B389" t="inlineStr">
         <is>
@@ -23401,7 +23401,7 @@
     </row>
     <row r="390">
       <c r="A390" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B390" t="inlineStr">
         <is>
@@ -23460,7 +23460,7 @@
     </row>
     <row r="391">
       <c r="A391" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B391" t="inlineStr">
         <is>
@@ -23519,7 +23519,7 @@
     </row>
     <row r="392">
       <c r="A392" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B392" t="inlineStr">
         <is>
@@ -23578,7 +23578,7 @@
     </row>
     <row r="393">
       <c r="A393" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B393" t="inlineStr">
         <is>
@@ -23637,7 +23637,7 @@
     </row>
     <row r="394">
       <c r="A394" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B394" t="inlineStr">
         <is>
@@ -23696,7 +23696,7 @@
     </row>
     <row r="395">
       <c r="A395" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B395" t="inlineStr">
         <is>
@@ -23755,7 +23755,7 @@
     </row>
     <row r="396">
       <c r="A396" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B396" t="inlineStr">
         <is>
@@ -23814,7 +23814,7 @@
     </row>
     <row r="397">
       <c r="A397" s="1" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B397" t="inlineStr">
         <is>
@@ -23873,7 +23873,7 @@
     </row>
     <row r="398">
       <c r="A398" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B398" t="inlineStr">
         <is>
@@ -23932,7 +23932,7 @@
     </row>
     <row r="399">
       <c r="A399" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B399" t="inlineStr">
         <is>
@@ -23991,7 +23991,7 @@
     </row>
     <row r="400">
       <c r="A400" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B400" t="inlineStr">
         <is>
@@ -24050,7 +24050,7 @@
     </row>
     <row r="401">
       <c r="A401" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B401" t="inlineStr">
         <is>
@@ -24109,7 +24109,7 @@
     </row>
     <row r="402">
       <c r="A402" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B402" t="inlineStr">
         <is>
@@ -24168,7 +24168,7 @@
     </row>
     <row r="403">
       <c r="A403" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B403" t="inlineStr">
         <is>
@@ -24227,7 +24227,7 @@
     </row>
     <row r="404">
       <c r="A404" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B404" t="inlineStr">
         <is>
@@ -24286,7 +24286,7 @@
     </row>
     <row r="405">
       <c r="A405" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B405" t="inlineStr">
         <is>
@@ -24345,7 +24345,7 @@
     </row>
     <row r="406">
       <c r="A406" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B406" t="inlineStr">
         <is>
@@ -24404,7 +24404,7 @@
     </row>
     <row r="407">
       <c r="A407" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B407" t="inlineStr">
         <is>
@@ -24463,7 +24463,7 @@
     </row>
     <row r="408">
       <c r="A408" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B408" t="inlineStr">
         <is>
@@ -24522,7 +24522,7 @@
     </row>
     <row r="409">
       <c r="A409" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B409" t="inlineStr">
         <is>
@@ -24581,7 +24581,7 @@
     </row>
     <row r="410">
       <c r="A410" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B410" t="inlineStr">
         <is>
@@ -24640,7 +24640,7 @@
     </row>
     <row r="411">
       <c r="A411" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B411" t="inlineStr">
         <is>
@@ -24699,7 +24699,7 @@
     </row>
     <row r="412">
       <c r="A412" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B412" t="inlineStr">
         <is>
@@ -24758,7 +24758,7 @@
     </row>
     <row r="413">
       <c r="A413" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B413" t="inlineStr">
         <is>
@@ -24817,7 +24817,7 @@
     </row>
     <row r="414">
       <c r="A414" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B414" t="inlineStr">
         <is>
@@ -24876,7 +24876,7 @@
     </row>
     <row r="415">
       <c r="A415" s="1" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B415" t="inlineStr">
         <is>
@@ -24935,7 +24935,7 @@
     </row>
     <row r="416">
       <c r="A416" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B416" t="inlineStr">
         <is>
@@ -24994,7 +24994,7 @@
     </row>
     <row r="417">
       <c r="A417" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B417" t="inlineStr">
         <is>
@@ -25053,7 +25053,7 @@
     </row>
     <row r="418">
       <c r="A418" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B418" t="inlineStr">
         <is>
@@ -25112,7 +25112,7 @@
     </row>
     <row r="419">
       <c r="A419" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B419" t="inlineStr">
         <is>
@@ -25171,7 +25171,7 @@
     </row>
     <row r="420">
       <c r="A420" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B420" t="inlineStr">
         <is>
@@ -25230,7 +25230,7 @@
     </row>
     <row r="421">
       <c r="A421" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B421" t="inlineStr">
         <is>
@@ -25289,7 +25289,7 @@
     </row>
     <row r="422">
       <c r="A422" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B422" t="inlineStr">
         <is>
@@ -25348,7 +25348,7 @@
     </row>
     <row r="423">
       <c r="A423" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B423" t="inlineStr">
         <is>
@@ -25407,7 +25407,7 @@
     </row>
     <row r="424">
       <c r="A424" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B424" t="inlineStr">
         <is>
@@ -25466,7 +25466,7 @@
     </row>
     <row r="425">
       <c r="A425" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B425" t="inlineStr">
         <is>
@@ -25525,7 +25525,7 @@
     </row>
     <row r="426">
       <c r="A426" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B426" t="inlineStr">
         <is>
@@ -25584,7 +25584,7 @@
     </row>
     <row r="427">
       <c r="A427" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B427" t="inlineStr">
         <is>
@@ -25643,7 +25643,7 @@
     </row>
     <row r="428">
       <c r="A428" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B428" t="inlineStr">
         <is>
@@ -25702,7 +25702,7 @@
     </row>
     <row r="429">
       <c r="A429" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B429" t="inlineStr">
         <is>
@@ -25761,7 +25761,7 @@
     </row>
     <row r="430">
       <c r="A430" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B430" t="inlineStr">
         <is>
@@ -25820,7 +25820,7 @@
     </row>
     <row r="431">
       <c r="A431" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B431" t="inlineStr">
         <is>
@@ -25879,7 +25879,7 @@
     </row>
     <row r="432">
       <c r="A432" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B432" t="inlineStr">
         <is>
@@ -25938,7 +25938,7 @@
     </row>
     <row r="433">
       <c r="A433" s="1" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B433" t="inlineStr">
         <is>

</xml_diff>